<commit_message>
update to disagreement df
</commit_message>
<xml_diff>
--- a/data/comments/icr4_disagreement.xlsx
+++ b/data/comments/icr4_disagreement.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M52"/>
+  <dimension ref="A1:N52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -362,60 +362,65 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>pers_exp_j</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>emot_exp_j</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>pol_opin_j</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>breadth_j</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>valence_j</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>contr_j</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>pers_exp_y</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>emot_exp_y</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>pol_opin_y</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>breadth_y</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>valence_y</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>contr_y</t>
         </is>
@@ -425,8 +430,10 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Zum Frühwarnsystem: ich wundere mich schon sehr lange. Wir schaffen es, zum Mond zu fliegen, aber Menschen, die in unser Land ohne Ausweispapiere einreisen wollen/Schutz suchen, die Fingerabdrücke abzunehmen und diese in einer zentralen Datei auszuwerten ist nicht möglich? Wie sollen Gefährder erkannt werden, wenn das System zu langsam und zu bürokratisch ist? Die Idee, ein Frühwarnsystem einzurichten ist gut, wird aber an den trägen Behörden scheitern. Mehr Personal: es ist noch nicht sehr lange her, da wurde die Reiterstaffel in Wuppertal abgeschafft, ebenso auch einige andere Staffeln. Das gab viel Leid, Tränen und Unverständnis. Und schon ein paar Jahre später werden neue Staffeln eingerichtet. Unsere Polizei schiebt Überstunden vor sich her, dass es einem graust. Nicht nur die Polizei muss verstärkt werden, sondern auch der Justizapparat. Um ein Gefühl der Sicherheit im Land zu haben, muss der Bürger sicher sein, dass nicht nur die Bombenleger, sondern auch die kleinen Einbrecher und Diebe gefasst und! verurteilt werden 3. : Gerne. Da so viele Menschen ihre Daten durch das Netz schicken, Payback- oder andere Karten nutzen und, und, und..glaube ich, dass sie Daten, die erfasst werden sollen, schon längst erfasst werden. 4.: Die Bundeswehr wird von den Steuerzahlern finanziert. Warum soll sie nicht unsere innere Sicherheit schützen? Also können Polizei und Bundeswehr miteinander üben. 5.: ja 6.: Es wäre gut, wenn innerhalb Deutschlands die Dateien vernetzt wären. Vielleicht erst einmal daran arbeiten.... 7. So schnell es geht 8.: Ist es das nicht schon bereits? 9.: Wir sind ein reiches Land und es geht uns sehr gut. Dass wir viele Flüchtlinge und/oder Asylsuchende hier haben, hat mich in meiner Lebensweise nicht eingeschränkt. Sobald aber ein Mensch, der hier die Gastfreundschaft genießt, straffällig wird ( damit meine ich nicht! das falsche Ausfüllen eines Formulars), hat er sein Gastrecht verwirkt und soll abgeschoben werden . Mein Fazit: Die einzelnen Punkte sind schön aufgestellt, aber leider sehe ich kein gutes Fundament. Wie konnte ein Amir die Behörden so lange an der Nase herumführen? Warum dauern Anträge manchmal Jahre? Um eine innere Sicherheit zu spüren müssen m. E. die Wege kurz und transparent sein. Polizei und Justiz müssen von Grund auf gestärkt werden. Ob mehr Abschiebungen alles rausreißen"? Ich weiß es nicht. Aber wenn die bestehenden Systeme stark wären, dann könnte man darauf auch aufbauen. Sonst ist der 9 Punkte Plan nur eine Worthülse.</t>
+        </is>
       </c>
       <c r="C2">
         <v>1</v>
@@ -435,16 +442,16 @@
         <v>1</v>
       </c>
       <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
         <v>6</v>
       </c>
-      <c r="F2">
-        <v>3</v>
-      </c>
       <c r="G2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2">
         <v>1</v>
@@ -453,12 +460,15 @@
         <v>1</v>
       </c>
       <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
         <v>5</v>
       </c>
-      <c r="L2">
-        <v>3</v>
-      </c>
       <c r="M2">
+        <v>3</v>
+      </c>
+      <c r="N2">
         <v>0</v>
       </c>
     </row>
@@ -466,23 +476,25 @@
       <c r="A3">
         <v>5</v>
       </c>
-      <c r="B3">
-        <v>0</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Erst einmal gut, dass man sich nicht nur auf eines versteift, sondern es mit vielen Maßnahmen angeht. Manche halte ich für mehr wichtig, manche für weniger. Vor allem aber muss man sehr früh ansetzen und ich denke das hat man erkannt. Denn wenn man früh ansetzt, die Gefährdung erkennt bzw. es am Ende durch eine gelungene Asyl-Politik dazu bringt, dass diese gar nicht entsteht, spart man sich auch die Kosten, um später Personen rund-um-die-Uhr zu überwachen. Bei der Thematik der Entschlüsselung der Netzkommunikation: Natürlich ist hier auch die Gefahr des Missbrauchs da, aber ich vertraue den staatlichen Stellen in gewisser Weise, wenngleich die Formulierung so klingt, als dauert so etwas ewig und man sei technisch gar nicht versiert. Wieso hat man dies nicht schon vorher gemacht? Forschung und Prävention ist schön und gut, aber nicht so relevant. Online-Waffenkauf halte ich auch nicht für so grundlegend und wichtig. Viel wichtiger ist da wieder die verstärkte Zusammenarbeit der Geheimdienste. Aber das verspricht man nach jedem Terror-Akt und am Ende bleibt jeder für sich. Ich verstehe ja auch die einzelnen Länder, die natürlich auch Informationen als Machtbasis für sich behalten wollen. Der Punkt mit den Abschiebung halte ich für sehr wichtig und ist daher an 9. Stelle etwas zu weit hinten platziert.</t>
+        </is>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
         <v>4</v>
       </c>
-      <c r="F3">
-        <v>3</v>
-      </c>
       <c r="G3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -491,15 +503,18 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
         <v>6</v>
       </c>
-      <c r="L3">
-        <v>3</v>
-      </c>
       <c r="M3">
+        <v>3</v>
+      </c>
+      <c r="N3">
         <v>0</v>
       </c>
     </row>
@@ -507,29 +522,31 @@
       <c r="A4">
         <v>7</v>
       </c>
-      <c r="B4">
-        <v>0</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>kann ich so nicht sehen. Wenn Asyl, dann mit Familie. Alles andere hat doch keine Sinn. Asylrecht ist doch ein Grundrecht bei uns. Da stellt sich die Frage nach Nutzen oder Schaden doch gar nicht. Wenn, dann müsste man grundsetzlich das Asylrecht in Frage stellen.</t>
+        </is>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -538,9 +555,12 @@
         <v>1</v>
       </c>
       <c r="L4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M4">
+        <v>2</v>
+      </c>
+      <c r="N4">
         <v>0</v>
       </c>
     </row>
@@ -548,40 +568,45 @@
       <c r="A5">
         <v>8</v>
       </c>
-      <c r="B5">
-        <v>0</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hallo zusammen. In meinen Augen ist dieser komplette Plan nutzlos . Er reagiert nur passive auf die aktuell stattfindenden Geschehnisse ohne auf die Wurzel der entstandenen Probleme einzugehen. Viele Punkte die hier aufgeführt sind stellen für den Bürger eine Schlechterstellung bei den Persönlichkeitsrechten dar. Außerdem finde ich es immer wieder bezeichnend das solche "Programme" immer vor einer Wahl gemacht werden. Was ist denn die letzten Jahre passiert ? Warum müssen dafür Programme gemacht werden. Die regierenden Parteien hatten mehr als genug Zeit die Ursachen abzustellen. Dafür braucht es keinen 9 Punkte Plan. Und was die Aussagen , gerade unserer Kanzlerin , wert sind kann man man aus ihrer Aussage zur "nationalen Anstrengung bei der Abschiebung " erkennen. Was ist daraus geworden ? Genau . Nichts. Ich gebe absolut nichts auf solche Programme weil es wie bei so vielen anderen Sachen an der Umsetzung hapern wird. Denn wie schon gesagt , nicht reden sondern machen ! Viele der Probleme hätten wir ohne die Entscheidung unserer Kanzlerin gar nicht.</t>
+        </is>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
         <v>4</v>
       </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
       <c r="G5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5">
         <v>1</v>
       </c>
       <c r="K5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M5">
+        <v>2</v>
+      </c>
+      <c r="N5">
         <v>1</v>
       </c>
     </row>
@@ -589,8 +614,10 @@
       <c r="A6">
         <v>9</v>
       </c>
-      <c r="B6">
-        <v>0</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>dann wirst du ein langes Leben haben</t>
+        </is>
       </c>
       <c r="C6">
         <v>0</v>
@@ -602,10 +629,10 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -620,9 +647,12 @@
         <v>0</v>
       </c>
       <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
         <v>4</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>0</v>
       </c>
     </row>
@@ -630,8 +660,10 @@
       <c r="A7">
         <v>10</v>
       </c>
-      <c r="B7">
-        <v>1</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ohne Familiennachzug scheitert eine Integration, jeder möchte doch zusammen mit seiner Familie leben. Was will einer alleine hier. So etwas wollte man doch selbst auch nicht.</t>
+        </is>
       </c>
       <c r="C7">
         <v>1</v>
@@ -643,27 +675,30 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7">
         <v>1</v>
       </c>
       <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
         <v>4</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>0</v>
       </c>
     </row>
@@ -671,40 +706,45 @@
       <c r="A8">
         <v>12</v>
       </c>
-      <c r="B8">
-        <v>0</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Also ich finde auch das die Bundeswehr im Inneren gegen das Gesetz verstoßen würde - das die Polizei eine bessere Ausrüstung benötigt ist auf alle Fälle klar! - die die unser Asylrecht missbrauchen, sollten sofort abgeschoben werden, damit andere die es benötigen, eher geholfen wird</t>
+        </is>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8">
         <v>2</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L8">
+        <v>2</v>
+      </c>
+      <c r="M8">
         <v>4</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>0</v>
       </c>
     </row>
@@ -712,40 +752,45 @@
       <c r="A9">
         <v>13</v>
       </c>
-      <c r="B9">
-        <v>0</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Wie gesagt sollte auch geändert werden. Oder sollen die Soldaten in Notsituationen einfach zugucken und nichts machen dürfen??</t>
+        </is>
       </c>
       <c r="C9">
         <v>0</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
       <c r="F9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9">
         <v>4</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>0</v>
       </c>
     </row>
@@ -753,23 +798,25 @@
       <c r="A10">
         <v>14</v>
       </c>
-      <c r="B10">
-        <v>0</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Punkt 4 (Bundeswehr) und Punkt 9 (Mehr Abschiebungen) halte ich für übertrieben. Die Forschungsvorhaben sollten nicht nur "**islamistischen** Terror" umfassen. Die Unterbindung des Online-Waffenhandels halte ich für sinnvoll.</t>
+        </is>
       </c>
       <c r="C10">
         <v>0</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F10">
         <v>3</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -781,12 +828,15 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L10">
         <v>3</v>
       </c>
       <c r="M10">
+        <v>3</v>
+      </c>
+      <c r="N10">
         <v>0</v>
       </c>
     </row>
@@ -794,40 +844,45 @@
       <c r="A11">
         <v>15</v>
       </c>
-      <c r="B11">
-        <v>0</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ich stimme dem 9 Punkteplan zu in allen Bereichen. Ich sage aber auch warum nicht stop mit den Asylaufnahmen.Wir sind kein Einwanderungsland. Warum nicht Schluss mit den aufnahmen. Das spart viel Kosten und Ärger.</t>
+        </is>
       </c>
       <c r="C11">
         <v>0</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11">
         <v>0</v>
       </c>
       <c r="J11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11">
         <v>1</v>
       </c>
       <c r="L11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M11">
+        <v>3</v>
+      </c>
+      <c r="N11">
         <v>1</v>
       </c>
     </row>
@@ -835,8 +890,10 @@
       <c r="A12">
         <v>16</v>
       </c>
-      <c r="B12">
-        <v>0</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Nicht immer nur reden und diskutieren, sondern einfach machen, umsetzen und ausprobieren, ggf. nachbessern. Es dauert einfach immer viel zu lange bzw. müssen leider Gottes immer erst ganz viele schlimme Dinge geschehen, bevor die Behörden mal entsprechende Gesetze oder Vorschriften auf den Weg bringen.</t>
+        </is>
       </c>
       <c r="C12">
         <v>0</v>
@@ -845,13 +902,13 @@
         <v>0</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -863,12 +920,15 @@
         <v>0</v>
       </c>
       <c r="K12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M12">
+        <v>2</v>
+      </c>
+      <c r="N12">
         <v>1</v>
       </c>
     </row>
@@ -876,8 +936,10 @@
       <c r="A13">
         <v>17</v>
       </c>
-      <c r="B13">
-        <v>0</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Dem kann ich nur zustimmen, zu den Schwierigkeiten der finanziellen Mittel und der schnellen reibungslosen Zusammenarbeit zwischen den Staaten sehe ich noch das Problem, dass es keine zeitlichen Vorgaben für die Durchführung des Planes gibt.</t>
+        </is>
       </c>
       <c r="C13">
         <v>0</v>
@@ -886,13 +948,13 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F13">
         <v>2</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -904,12 +966,15 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M13">
+        <v>3</v>
+      </c>
+      <c r="N13">
         <v>0</v>
       </c>
     </row>
@@ -917,29 +982,31 @@
       <c r="A14">
         <v>18</v>
       </c>
-      <c r="B14">
-        <v>0</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Der 9. Punkte Plan hört sich geschrieben schon mal gut an. Nur will Merkel diesen tatsächlich realisiere?! Daran möchte ich zweifeln. Selbst wenn man diese Frau bei Debatten beobachtet, sie kann sich ja toll überall heraus reden und meint alles wird gut! Für wen? Nicht für das Volk. In ihren Augen hingegen sind Zweifel und Unsicherheit über ihre eigenen Worte zu sehen! Gegen wie viele Gesetze hat diese Frau schon verstoßen?! Für mich ist diese Person, die ehemals zu Zeiten der DDR bei der Stasi war nicht glaubwürdig und für das "DEUTSCHE VOLK" untragbar. Doch ich fürchte, sie wird weiterhin Kanzlerin bleiben! Dafür gibt es so, wie Medien berichten leider noch immer genug Menschen, die ihr vertrauen. Wenn ich hundertmal betrogen werde, vertraue ich nicht mehr.</t>
+        </is>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14">
         <v>1</v>
       </c>
       <c r="E14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14">
         <v>1</v>
@@ -948,9 +1015,12 @@
         <v>1</v>
       </c>
       <c r="L14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M14">
+        <v>3</v>
+      </c>
+      <c r="N14">
         <v>1</v>
       </c>
     </row>
@@ -958,8 +1028,10 @@
       <c r="A15">
         <v>19</v>
       </c>
-      <c r="B15">
-        <v>0</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Grundsätzlich halte ich es für sehr sinnvoll die gemachten Erfahrungen von Migration in unser Land zu nutzen und viel breiter zu diskutieren. Wirtschaftliche Interessen zu benennen und notwendige Partizipation zu diskutieren. Wenn Angst/Kontrolle vorherrscht sind die Kinder in den Brunnen gefallen....Leider ist die Sicht der Flüchtlingswelle aus 2015 so abgelegt. Sich aufzustellen gegen Terrorismus bedeutet eine sehr feinfühlige Balance zwischen empfundenen Schutz und der Lust auf ein freies und selbstbestimmtes Leben....</t>
+        </is>
       </c>
       <c r="C15">
         <v>0</v>
@@ -968,13 +1040,13 @@
         <v>0</v>
       </c>
       <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
         <v>4</v>
       </c>
-      <c r="F15">
-        <v>3</v>
-      </c>
       <c r="G15">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -983,15 +1055,18 @@
         <v>0</v>
       </c>
       <c r="J15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15">
+        <v>1</v>
+      </c>
+      <c r="L15">
         <v>4</v>
       </c>
-      <c r="L15">
-        <v>3</v>
-      </c>
       <c r="M15">
+        <v>3</v>
+      </c>
+      <c r="N15">
         <v>0</v>
       </c>
     </row>
@@ -999,8 +1074,10 @@
       <c r="A16">
         <v>20</v>
       </c>
-      <c r="B16">
-        <v>0</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Auf dem Papier klingt der Plan gut, aber wie immer wird es auf die konkrete Umsetzung ankommen.</t>
+        </is>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1012,10 +1089,10 @@
         <v>0</v>
       </c>
       <c r="F16">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H16">
         <v>0</v>
@@ -1030,9 +1107,12 @@
         <v>0</v>
       </c>
       <c r="L16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M16">
+        <v>1</v>
+      </c>
+      <c r="N16">
         <v>0</v>
       </c>
     </row>
@@ -1040,26 +1120,28 @@
       <c r="A17">
         <v>27</v>
       </c>
-      <c r="B17">
-        <v>0</v>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>diese 9 punkte plan funktioniert nur, in dem man im nahen osten die länder von terorgruppen befreit und nicht durch waffenverkäufe unterstützt. diese terorangriffe sind vom westen mitverantwortlich.</t>
+        </is>
       </c>
       <c r="C17">
         <v>0</v>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17">
+        <v>2</v>
+      </c>
+      <c r="G17">
         <v>4</v>
       </c>
-      <c r="G17">
-        <v>1</v>
-      </c>
       <c r="H17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17">
         <v>0</v>
@@ -1068,12 +1150,15 @@
         <v>0</v>
       </c>
       <c r="K17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L17">
+        <v>2</v>
+      </c>
+      <c r="M17">
         <v>4</v>
       </c>
-      <c r="M17">
+      <c r="N17">
         <v>1</v>
       </c>
     </row>
@@ -1081,40 +1166,45 @@
       <c r="A18">
         <v>35</v>
       </c>
-      <c r="B18">
-        <v>0</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ich finde es erschreckend, wenn größere Veranstaltungen nur noch mit massiven Sperren gegen Fahrzeuganschläge und körperliche Durchsuchungen möglich sind. Da bleibe ich lieber Zuhause.</t>
+        </is>
       </c>
       <c r="C18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F18">
         <v>2</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H18">
         <v>0</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L18">
+        <v>2</v>
+      </c>
+      <c r="M18">
         <v>4</v>
       </c>
-      <c r="M18">
+      <c r="N18">
         <v>0</v>
       </c>
     </row>
@@ -1122,8 +1212,10 @@
       <c r="A19">
         <v>43</v>
       </c>
-      <c r="B19">
-        <v>0</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Meiner Meinung nach gibt es nichts zu Ergänzen, aber die Punkte müssen schnellst möglich durchgesetz werde. und das ist in unserem Land ein grpßes Problem. Viel Reden, wenig Durchführung.</t>
+        </is>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1135,10 +1227,10 @@
         <v>0</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H19">
         <v>0</v>
@@ -1153,9 +1245,12 @@
         <v>0</v>
       </c>
       <c r="L19">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M19">
+        <v>3</v>
+      </c>
+      <c r="N19">
         <v>1</v>
       </c>
     </row>
@@ -1163,40 +1258,45 @@
       <c r="A20">
         <v>44</v>
       </c>
-      <c r="B20">
-        <v>0</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Wird nur funktionieren wenn der 9-Punkte-Plan auch genauso angewendet wird. Ergänzend würde ich sagen, dass strafällige gewordene Flüchtlinge mit sofortiger Wirkung abgeschoben werden und nicht erst nach Monaten egal Krankheit, etc vorliegt.</t>
+        </is>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20">
         <v>1</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20">
         <v>0</v>
       </c>
       <c r="J20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20">
         <v>1</v>
       </c>
       <c r="L20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M20">
+        <v>2</v>
+      </c>
+      <c r="N20">
         <v>1</v>
       </c>
     </row>
@@ -1204,40 +1304,45 @@
       <c r="A21">
         <v>46</v>
       </c>
-      <c r="B21">
-        <v>1</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tatsächlich hatte ich noch keinen direkten Kontakt, aber bei Großveranstaltungen nimmt man die Gefahr mittelbar durch sehr konsequente Personenkontrollen war. Und an zentralen, belebten Orten kommt schon mal der Gedanke auf, "was wäre wenn.....".</t>
+        </is>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
       <c r="E21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21">
         <v>0</v>
       </c>
       <c r="K21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21">
         <v>4</v>
       </c>
-      <c r="M21">
+      <c r="N21">
         <v>0</v>
       </c>
     </row>
@@ -1245,40 +1350,45 @@
       <c r="A22">
         <v>48</v>
       </c>
-      <c r="B22">
-        <v>0</v>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Ein Plan mag ja gut und schön sein, aber es sollten auch Dinge umgesetzt werden. Bei vielen Dingen habe ich nur das Gefühl, das viel drüber gesprochen wird. Aber wird auch was umgesetzt? Ich meine, warum muss man erst Monate über Namen diskutieren, über Dinge die dann vielleicht a) nie so umgesetzt werden oder b) wenn sie Zustande kommen, irgendwie ganz anders. Siehe z.b. die Erst Aufnahme Stellen. Mein Gott, was wurde da damals über die verschieden Namen geredet, bevor es überhaupt eine gab. Warum muss es Gastarbeiter, Ausländer, Migrant oder was weiß ich heißen? Der Name ändert nichts, der Name macht es nicht besser und nur weil mich sich schöne Namen ausdenkt oder Pläne, heißt das nicht, das die Problematik dadurch aufhört. Waffenverkäufe sind doch echt sinnlos an andere Länder, Hunger, Krieg... das muss gestoppt werden</t>
+        </is>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22">
         <v>1</v>
       </c>
       <c r="E22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L22">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M22">
+        <v>3</v>
+      </c>
+      <c r="N22">
         <v>1</v>
       </c>
     </row>
@@ -1286,24 +1396,26 @@
       <c r="A23">
         <v>57</v>
       </c>
-      <c r="B23">
-        <v>0</v>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Intensivere Zusammenarbeit mit Tourismusexperten. Es hat sich gezeigt, dass die beiden Begriffe Terrorismusexperte und Tourismusexperte nicht nur bei den Buchstaben eng beieinanderliegen, sondern auch was die Auswahl der Ziele von Anschlägen betrifft, dies waren vorwiegend Ziele, die ich erst kurz zuvor selbst als Tourist besucht hatte oder welche ich geplant hatte, zu besuchen. Man muss also schauen, welche Destinationen sind touristisch interessant, welche Region boomt usw. d.h. überlegen, wie kann ein Terrorist einem Gebiet auch wirtschaftlich den größtmöglichen Schaden zufügen (durch ausbleibende Touristen usw.) und diese identifizierten Ziele dann intensiver observieren und schützen.</t>
+        </is>
       </c>
       <c r="C23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F23">
+        <v>2</v>
+      </c>
+      <c r="G23">
         <v>4</v>
       </c>
-      <c r="G23">
-        <v>0</v>
-      </c>
       <c r="H23">
         <v>0</v>
       </c>
@@ -1314,12 +1426,15 @@
         <v>0</v>
       </c>
       <c r="K23">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L23">
+        <v>2</v>
+      </c>
+      <c r="M23">
         <v>4</v>
       </c>
-      <c r="M23">
+      <c r="N23">
         <v>0</v>
       </c>
     </row>
@@ -1327,40 +1442,45 @@
       <c r="A24">
         <v>59</v>
       </c>
-      <c r="B24">
-        <v>0</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Terroristen dürfen nicht abgeschoben werden, denn in dem Abgeschobenen Land könnten sie auch Menschen töten. Die Leute haben jeden Respeckt vor dem Leben verloren und müßen unschädlich gemacht werden!</t>
+        </is>
       </c>
       <c r="C24">
         <v>0</v>
       </c>
       <c r="D24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24">
         <v>2</v>
       </c>
       <c r="G24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24">
         <v>0</v>
       </c>
       <c r="J24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24">
         <v>1</v>
       </c>
       <c r="L24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M24">
+        <v>2</v>
+      </c>
+      <c r="N24">
         <v>1</v>
       </c>
     </row>
@@ -1368,8 +1488,10 @@
       <c r="A25">
         <v>64</v>
       </c>
-      <c r="B25">
-        <v>0</v>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Diese Punkte sind gut und richtig, nur viel zu spät beschlossen und noch lange nicht umgesetzt. Das Kompetenzgerangel über die Dienste -Geheimdienst, Nachrichtendienst, Polizei und Politik hat noch gar nicht begonnen. Einer will dem anderen "Seine Erkenntnisse" nicht zur Verfügung stellen usw. Dazu kommt die Bundestagswahl ! Bei größeren Veränderungen, eventuell neuen Kanzler, müssen die Ausschüsse neu gewählt und besetzt werden. Bis da positive Ergebnisse greifen, schreiben wir das Frühjahr 2018. Und die Gefährter lachen sich schlapp und bomben weiter.</t>
+        </is>
       </c>
       <c r="C25">
         <v>0</v>
@@ -1378,13 +1500,13 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F25">
         <v>3</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H25">
         <v>0</v>
@@ -1396,12 +1518,15 @@
         <v>0</v>
       </c>
       <c r="K25">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L25">
         <v>3</v>
       </c>
       <c r="M25">
+        <v>3</v>
+      </c>
+      <c r="N25">
         <v>1</v>
       </c>
     </row>
@@ -1409,23 +1534,25 @@
       <c r="A26">
         <v>65</v>
       </c>
-      <c r="B26">
-        <v>0</v>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>niemand ist Weltpolizei aber einige Länder benehmen sich so ich denke es nicht unsee Aufgabe in der Welt mit Gewalt einzuwirken und leider ist es wohl -viel- zu spät</t>
+        </is>
       </c>
       <c r="C26">
         <v>0</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26">
         <v>2</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H26">
         <v>0</v>
@@ -1437,12 +1564,15 @@
         <v>0</v>
       </c>
       <c r="K26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L26">
         <v>2</v>
       </c>
       <c r="M26">
+        <v>2</v>
+      </c>
+      <c r="N26">
         <v>0</v>
       </c>
     </row>
@@ -1450,29 +1580,31 @@
       <c r="A27">
         <v>69</v>
       </c>
-      <c r="B27">
-        <v>0</v>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Gefährdet zu überwachen dürfte schwierig sein.Ich bin der Meinung, daß alle Verdächtigen sofort unser Land verlassen müssten.Aber das ist vielleicht nicht immer möglich.Aber die Gefahr bleibt immer bestehen,wir wissen nie genau,wie Gefährder ticken und wann und wie sie aktiv werden.</t>
+        </is>
       </c>
       <c r="C27">
         <v>0</v>
       </c>
       <c r="D27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27">
         <v>1</v>
       </c>
       <c r="F27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H27">
         <v>0</v>
       </c>
       <c r="I27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J27">
         <v>1</v>
@@ -1481,9 +1613,12 @@
         <v>1</v>
       </c>
       <c r="L27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M27">
+        <v>2</v>
+      </c>
+      <c r="N27">
         <v>1</v>
       </c>
     </row>
@@ -1491,40 +1626,45 @@
       <c r="A28">
         <v>71</v>
       </c>
-      <c r="B28">
-        <v>0</v>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Ersteinmal müßte Weltweit jeder Krieg beendet werden und alle Religionen verboten werden um keinen neuen Hass zu erzeugen. Nur ausreichende Bildung schützt vor hasserfüllter Beeinflussung. Wenn die Flüchtlinge sich nicht in den geflüchteten Staaten an deren Lebensweise anpassen wollen haben Sie in diesen nicht verloren!</t>
+        </is>
       </c>
       <c r="C28">
         <v>0</v>
       </c>
       <c r="D28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28">
         <v>0</v>
       </c>
       <c r="J28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28">
+        <v>1</v>
+      </c>
+      <c r="L28">
         <v>4</v>
       </c>
-      <c r="L28">
-        <v>2</v>
-      </c>
       <c r="M28">
+        <v>2</v>
+      </c>
+      <c r="N28">
         <v>1</v>
       </c>
     </row>
@@ -1532,8 +1672,10 @@
       <c r="A29">
         <v>72</v>
       </c>
-      <c r="B29">
-        <v>0</v>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>wenn man die Kontrollen mal erst nimmt. Ja zu wenig Polizei, aber selber Schuld, lieber das Geld für unütze Dinge ausgeben.</t>
+        </is>
       </c>
       <c r="C29">
         <v>0</v>
@@ -1542,16 +1684,16 @@
         <v>0</v>
       </c>
       <c r="E29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F29">
         <v>2</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29">
         <v>0</v>
@@ -1560,12 +1702,15 @@
         <v>0</v>
       </c>
       <c r="K29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L29">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M29">
+        <v>2</v>
+      </c>
+      <c r="N29">
         <v>1</v>
       </c>
     </row>
@@ -1573,40 +1718,45 @@
       <c r="A30">
         <v>73</v>
       </c>
-      <c r="B30">
-        <v>0</v>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Ich finde es gut, dass Frau Merkel und ihre Mitarbeiter sich intensiv zusammensetzen und einen Umfassenden Plan erstellen - allerdings sind manche der Punkte eher schwammig, schwer umsetzbar und schlicht ein "Über das Ziel Hinausschießen" - wenn es zum Beispiel darum geht, generell stärker online Kommunikation zu überwachen, ist das ein massiver Übergriff auf die Privatsphäre der Bürger - denn dann müsste das bedeuten, dass konkret ALLE Nutzer "abgehorcht" werden - anderenfalls ist es eine klare Marginalisierung und Diskriminierung bestimmter Ethnischer Gruppierungen und steht mehr für Rassismus denn für die gepredigte europäische/deutsche Offenheit, Toleranz, Vorurteilsfreiheit.</t>
+        </is>
       </c>
       <c r="C30">
         <v>0</v>
       </c>
       <c r="D30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E30">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F30">
         <v>3</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H30">
         <v>0</v>
       </c>
       <c r="I30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J30">
         <v>1</v>
       </c>
       <c r="K30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M30">
+        <v>3</v>
+      </c>
+      <c r="N30">
         <v>0</v>
       </c>
     </row>
@@ -1614,40 +1764,45 @@
       <c r="A31">
         <v>77</v>
       </c>
-      <c r="B31">
-        <v>0</v>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Der Terror lässt sich nicht wirklich stoppen.Die Vergangenheit hat gezeigt das es nicht wirklich klappt.Diktatoren geben sich die Klinke in die Hand.Und wenn sie dann doch mal gestürtzt werden dann nehmen radikale Kräfte den Platz ein. Bestes Beispiel damals Saddam Hussein.Hätte man den damals an der Macht gelassen wäre der IS vielleicht gar nicht so hoch gekommen. Unter Saddam ging es den Menschen bestimmt nicht schlechter als jetzt. Kriege haben jedenfalls selten zu Frieden geführt.Es sind doch im Prinzip immer die selben Gegenden in denen Krieg herscht.Vielleicht sollte man aufhören sich überall kriegerisch zu beteiligen,was vorallem auf die USA und Russland zutrifft. Manchmal hat man das Gefühl die bekämpfen sich gegenseitig und die Länder in dem sie das tun müssen leiden.</t>
+        </is>
       </c>
       <c r="C31">
         <v>0</v>
       </c>
       <c r="D31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31">
         <v>2</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31">
         <v>0</v>
       </c>
       <c r="J31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L31">
         <v>2</v>
       </c>
       <c r="M31">
+        <v>2</v>
+      </c>
+      <c r="N31">
         <v>0</v>
       </c>
     </row>
@@ -1655,8 +1810,10 @@
       <c r="A32">
         <v>79</v>
       </c>
-      <c r="B32">
-        <v>0</v>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Klare Kontrolle der zuwanderung, überwachung von risikogruppen und endlich öffendliches eingeständnis das es sehr wohl innerhalb gewisser gruppen eine affinität zur gewalt gibt</t>
+        </is>
       </c>
       <c r="C32">
         <v>0</v>
@@ -1665,16 +1822,16 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F32">
         <v>2</v>
       </c>
       <c r="G32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32">
         <v>0</v>
@@ -1683,12 +1840,15 @@
         <v>0</v>
       </c>
       <c r="K32">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L32">
+        <v>2</v>
+      </c>
+      <c r="M32">
         <v>4</v>
       </c>
-      <c r="M32">
+      <c r="N32">
         <v>0</v>
       </c>
     </row>
@@ -1696,40 +1856,45 @@
       <c r="A33">
         <v>80</v>
       </c>
-      <c r="B33">
-        <v>1</v>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Ich habe zum Glück noch keine persönlichen Erfahrungen mit Terror gemacht. Aber ich habe Verwandte in Berlin, und als das Attentat auf dem Weihnachtsmarkt im Dezember 2016 passierte, war ich sehr besorgt und vollkommen verängstigt. Man steht so fassungslos demgegenüber und kann nichts machen. Zum Glück waren meine Verwandten nicht betroffen, aber die Angst saß tief. Ich habe jetzt immer Bedenken,wo sich große Menschenmengen aufhalten und versuche, sie zu vermeiden. Aber das ist auch nicht immer möglich. Großveranstaltungen machen mir Angst.</t>
+        </is>
       </c>
       <c r="C33">
         <v>1</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G33">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I33">
         <v>1</v>
       </c>
       <c r="J33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L33">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M33">
+        <v>3</v>
+      </c>
+      <c r="N33">
         <v>0</v>
       </c>
     </row>
@@ -1737,8 +1902,10 @@
       <c r="A34">
         <v>92</v>
       </c>
-      <c r="B34">
-        <v>0</v>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Terror wird es immer geben, aber nicht in diesem Maße. Gefärder gehören besser überwacht, Grenzen besser kontrolliert, und die Einreisungen eingeschränkt. Aber auch dann wird es leider immer Terror geben, weil es einfach kranke Menschen auf dieser Welt gibt.</t>
+        </is>
       </c>
       <c r="C34">
         <v>0</v>
@@ -1747,13 +1914,13 @@
         <v>0</v>
       </c>
       <c r="E34">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F34">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G34">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H34">
         <v>0</v>
@@ -1765,12 +1932,15 @@
         <v>0</v>
       </c>
       <c r="K34">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L34">
         <v>2</v>
       </c>
       <c r="M34">
+        <v>2</v>
+      </c>
+      <c r="N34">
         <v>0</v>
       </c>
     </row>
@@ -1778,8 +1948,10 @@
       <c r="A35">
         <v>96</v>
       </c>
-      <c r="B35">
-        <v>0</v>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Ich finde den 9-Punkte -Plan sehr aufschlussreich. Aber so ganz neu ist er ja nicht. Inzwischen ist ja schon eine Zeit vergangen und ich sehe da einen großen Handlungsbedarf, wenn der Plan eingehalten werden soll!!!!</t>
+        </is>
       </c>
       <c r="C35">
         <v>0</v>
@@ -1791,27 +1963,30 @@
         <v>0</v>
       </c>
       <c r="F35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H35">
         <v>0</v>
       </c>
       <c r="I35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K35">
         <v>0</v>
       </c>
       <c r="L35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M35">
+        <v>1</v>
+      </c>
+      <c r="N35">
         <v>0</v>
       </c>
     </row>
@@ -1819,8 +1994,10 @@
       <c r="A36">
         <v>97</v>
       </c>
-      <c r="B36">
-        <v>0</v>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>**Die Regierung sollte mehr für die Früherkennung und Integration tun. Überwachung schürrt nur mehr Misstrauen und schränkt die Freiheitsrechte der Bürger ziemlich ein.** Mit Abschiebung ist das Problem ebenfalls nicht gelöst, sondern wird nur etwas rausgezögert. Panik und Angst ist zudem ein sehr schlechter Berater.</t>
+        </is>
       </c>
       <c r="C36">
         <v>0</v>
@@ -1829,13 +2006,13 @@
         <v>0</v>
       </c>
       <c r="E36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F36">
         <v>3</v>
       </c>
       <c r="G36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H36">
         <v>0</v>
@@ -1847,12 +2024,15 @@
         <v>0</v>
       </c>
       <c r="K36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L36">
+        <v>3</v>
+      </c>
+      <c r="M36">
         <v>4</v>
       </c>
-      <c r="M36">
+      <c r="N36">
         <v>0</v>
       </c>
     </row>
@@ -1860,23 +2040,25 @@
       <c r="A37">
         <v>99</v>
       </c>
-      <c r="B37">
-        <v>0</v>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Terror müssen wir an der Wurzel bekämpfen. Konfliktlösungen suchen, vermitteln. Weiterhin. Keine Waffen senden, keine Unterstützung geben.</t>
+        </is>
       </c>
       <c r="C37">
         <v>0</v>
       </c>
       <c r="D37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F37">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G37">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H37">
         <v>0</v>
@@ -1888,12 +2070,15 @@
         <v>0</v>
       </c>
       <c r="K37">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L37">
+        <v>2</v>
+      </c>
+      <c r="M37">
         <v>4</v>
       </c>
-      <c r="M37">
+      <c r="N37">
         <v>0</v>
       </c>
     </row>
@@ -1901,23 +2086,25 @@
       <c r="A38">
         <v>106</v>
       </c>
-      <c r="B38">
-        <v>1</v>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Wir müssen potenziellen Gefährdern auch die Möglichkeit geben, von selbst auszusteigen. Für die rechte Szene gibt es zum Beispiel das Programm "Exit", das eben auch Schutz vor den alten "Freunden" verspricht, sowas sollten wir auch für islamischen Terror in Erwägung ziehen. Außerdem sollten wir endlich anfangen, Integration zu leben. Hier muss der Staat aber auch wieder mehr in die Gemeinden und ihre Angebote investieren (Jugendtreffs, Kulturveranstaltungen). So kann ich eventuell Jugendliche abfangen, bevor sie radikalisiert werden!</t>
+        </is>
       </c>
       <c r="C38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38">
         <v>0</v>
       </c>
       <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
         <v>4</v>
       </c>
-      <c r="F38">
-        <v>3</v>
-      </c>
       <c r="G38">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H38">
         <v>0</v>
@@ -1929,12 +2116,15 @@
         <v>0</v>
       </c>
       <c r="K38">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L38">
         <v>4</v>
       </c>
       <c r="M38">
+        <v>4</v>
+      </c>
+      <c r="N38">
         <v>0</v>
       </c>
     </row>
@@ -1942,26 +2132,28 @@
       <c r="A39">
         <v>111</v>
       </c>
-      <c r="B39">
-        <v>0</v>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Korrekt. Hauptsächlich um abtrünnige Wähler von der AFD/Themen zurückzuholen.</t>
+        </is>
       </c>
       <c r="C39">
         <v>0</v>
       </c>
       <c r="D39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E39">
         <v>1</v>
       </c>
       <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39">
         <v>4</v>
       </c>
-      <c r="G39">
-        <v>1</v>
-      </c>
       <c r="H39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I39">
         <v>0</v>
@@ -1970,12 +2162,15 @@
         <v>0</v>
       </c>
       <c r="K39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L39">
+        <v>1</v>
+      </c>
+      <c r="M39">
         <v>4</v>
       </c>
-      <c r="M39">
+      <c r="N39">
         <v>1</v>
       </c>
     </row>
@@ -1983,8 +2178,10 @@
       <c r="A40">
         <v>112</v>
       </c>
-      <c r="B40">
-        <v>0</v>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Hallo Herr Bartsch Ihr Vorschlag hört sich ja erst einmal ganz gut und begrüßenswert an, wie darf ich mir denn Ihren "sozialen Aufbruch" so vorstellen...?!?</t>
+        </is>
       </c>
       <c r="C40">
         <v>0</v>
@@ -1993,30 +2190,33 @@
         <v>0</v>
       </c>
       <c r="E40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G40">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H40">
         <v>0</v>
       </c>
       <c r="I40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L40">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M40">
+        <v>3</v>
+      </c>
+      <c r="N40">
         <v>0</v>
       </c>
     </row>
@@ -2024,8 +2224,10 @@
       <c r="A41">
         <v>113</v>
       </c>
-      <c r="B41">
-        <v>0</v>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Jeder sollte seine Meinung haben und diese auch aussprechen dürfen, aber den anderen für seine Meinung nicht verurteilen. Respekt und Toleranz spielen da eine große Rolle. Religionen sollten auch nicht dafür genutzt werden, Menschen zu verhetzen, um anderen Menschen wiederum Schmerz und Leid zuzufügen.</t>
+        </is>
       </c>
       <c r="C41">
         <v>0</v>
@@ -2034,13 +2236,13 @@
         <v>0</v>
       </c>
       <c r="E41">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F41">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H41">
         <v>0</v>
@@ -2052,12 +2254,15 @@
         <v>0</v>
       </c>
       <c r="K41">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M41">
+        <v>1</v>
+      </c>
+      <c r="N41">
         <v>0</v>
       </c>
     </row>
@@ -2065,8 +2270,10 @@
       <c r="A42">
         <v>119</v>
       </c>
-      <c r="B42">
-        <v>0</v>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Solange sich die sogenannten Großmächte dieser Welt in alles einmischen, was sie nichts angeht, wird der Terror weitergehen!!!</t>
+        </is>
       </c>
       <c r="C42">
         <v>0</v>
@@ -2075,30 +2282,33 @@
         <v>0</v>
       </c>
       <c r="E42">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F42">
         <v>2</v>
       </c>
       <c r="G42">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H42">
         <v>0</v>
       </c>
       <c r="I42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J42">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K42">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L42">
         <v>2</v>
       </c>
       <c r="M42">
+        <v>2</v>
+      </c>
+      <c r="N42">
         <v>0</v>
       </c>
     </row>
@@ -2106,26 +2316,28 @@
       <c r="A43">
         <v>122</v>
       </c>
-      <c r="B43">
-        <v>0</v>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Meiner Meinung nach kann das Problem hauptsächlich nur an der Wurzel bekämpft werden - sprich in den Ländern in denen der Terror entsteht und von da aus in die Welt getragen wird. Dort muss man verstärkt anpacken - Aufklärung leisten - Hilfen anbieten. Sind die Typen erstmal radikalisiert gibt's nimmer viel zurück...</t>
+        </is>
       </c>
       <c r="C43">
         <v>0</v>
       </c>
       <c r="D43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G43">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I43">
         <v>0</v>
@@ -2134,12 +2346,15 @@
         <v>0</v>
       </c>
       <c r="K43">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L43">
+        <v>2</v>
+      </c>
+      <c r="M43">
         <v>4</v>
       </c>
-      <c r="M43">
+      <c r="N43">
         <v>0</v>
       </c>
     </row>
@@ -2147,8 +2362,10 @@
       <c r="A44">
         <v>126</v>
       </c>
-      <c r="B44">
-        <v>0</v>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Der 9-Punkte Plan wäre nicht schlecht... er müsste nur umgesetzt werden. Klar, man braucht erst einen Plan bevor man handelt, doch wird hier in Deutschland zu lange diskutiert wie man vorgeht, Handlung erfolgt zu spät.</t>
+        </is>
       </c>
       <c r="C44">
         <v>0</v>
@@ -2157,13 +2374,13 @@
         <v>0</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F44">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G44">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H44">
         <v>0</v>
@@ -2178,9 +2395,12 @@
         <v>0</v>
       </c>
       <c r="L44">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M44">
+        <v>3</v>
+      </c>
+      <c r="N44">
         <v>0</v>
       </c>
     </row>
@@ -2188,8 +2408,10 @@
       <c r="A45">
         <v>127</v>
       </c>
-      <c r="B45">
-        <v>0</v>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Ich halte den Plan für einen moderaten Fortschritt und der Sicherheitslage für angemessen.</t>
+        </is>
       </c>
       <c r="C45">
         <v>0</v>
@@ -2198,13 +2420,13 @@
         <v>0</v>
       </c>
       <c r="E45">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F45">
         <v>1</v>
       </c>
       <c r="G45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H45">
         <v>0</v>
@@ -2219,9 +2441,12 @@
         <v>0</v>
       </c>
       <c r="L45">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M45">
+        <v>1</v>
+      </c>
+      <c r="N45">
         <v>0</v>
       </c>
     </row>
@@ -2229,40 +2454,45 @@
       <c r="A46">
         <v>134</v>
       </c>
-      <c r="B46">
-        <v>0</v>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Das sind alles Punkte die ich wichtig finde, aber ich glaube nicht im geringsten daran, dass überhaupt etwas davon von Frau Merkel umgesetzt werden kann oder wird</t>
+        </is>
       </c>
       <c r="C46">
         <v>0</v>
       </c>
       <c r="D46">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E46">
         <v>1</v>
       </c>
       <c r="F46">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H46">
         <v>0</v>
       </c>
       <c r="I46">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J46">
         <v>1</v>
       </c>
       <c r="K46">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L46">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M46">
+        <v>2</v>
+      </c>
+      <c r="N46">
         <v>0</v>
       </c>
     </row>
@@ -2270,8 +2500,10 @@
       <c r="A47">
         <v>137</v>
       </c>
-      <c r="B47">
-        <v>0</v>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Geht in Ordnung</t>
+        </is>
       </c>
       <c r="C47">
         <v>0</v>
@@ -2283,11 +2515,11 @@
         <v>0</v>
       </c>
       <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47">
         <v>4</v>
       </c>
-      <c r="G47">
-        <v>0</v>
-      </c>
       <c r="H47">
         <v>0</v>
       </c>
@@ -2301,9 +2533,12 @@
         <v>0</v>
       </c>
       <c r="L47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M47">
+        <v>1</v>
+      </c>
+      <c r="N47">
         <v>0</v>
       </c>
     </row>
@@ -2311,40 +2546,45 @@
       <c r="A48">
         <v>144</v>
       </c>
-      <c r="B48">
-        <v>0</v>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Fachkräftemangel? Sie glauben nicht wirklich an dieses Ammenmärchen??? Hoffentlich glauben Sie nicht, dass wir 2,5 Mil. Arbeitslose haben. Falls doch, haben die Politiker ihr Ziel leider erreicht.</t>
+        </is>
       </c>
       <c r="C48">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D48">
         <v>1</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F48">
         <v>2</v>
       </c>
       <c r="G48">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I48">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K48">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L48">
         <v>2</v>
       </c>
       <c r="M48">
+        <v>2</v>
+      </c>
+      <c r="N48">
         <v>1</v>
       </c>
     </row>
@@ -2352,8 +2592,10 @@
       <c r="A49">
         <v>147</v>
       </c>
-      <c r="B49">
-        <v>0</v>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Ich frage mich warum diese Punkte nicht schon lange umgesetzt sind, es wird einfach immer wieder viel zu viel diskutiert.</t>
+        </is>
       </c>
       <c r="C49">
         <v>0</v>
@@ -2365,10 +2607,10 @@
         <v>0</v>
       </c>
       <c r="F49">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G49">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H49">
         <v>0</v>
@@ -2383,9 +2625,12 @@
         <v>0</v>
       </c>
       <c r="L49">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M49">
+        <v>2</v>
+      </c>
+      <c r="N49">
         <v>0</v>
       </c>
     </row>
@@ -2393,8 +2638,10 @@
       <c r="A50">
         <v>148</v>
       </c>
-      <c r="B50">
-        <v>0</v>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Gut das ist</t>
+        </is>
       </c>
       <c r="C50">
         <v>0</v>
@@ -2406,11 +2653,11 @@
         <v>0</v>
       </c>
       <c r="F50">
+        <v>0</v>
+      </c>
+      <c r="G50">
         <v>4</v>
       </c>
-      <c r="G50">
-        <v>0</v>
-      </c>
       <c r="H50">
         <v>0</v>
       </c>
@@ -2424,9 +2671,12 @@
         <v>0</v>
       </c>
       <c r="L50">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M50">
+        <v>1</v>
+      </c>
+      <c r="N50">
         <v>0</v>
       </c>
     </row>
@@ -2434,8 +2684,10 @@
       <c r="A51">
         <v>149</v>
       </c>
-      <c r="B51">
-        <v>0</v>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Ich glaube nicht, das dies geht. Ich wüssste auch nicht wie man dem Terror entgegen treten könnte.</t>
+        </is>
       </c>
       <c r="C51">
         <v>0</v>
@@ -2444,14 +2696,14 @@
         <v>0</v>
       </c>
       <c r="E51">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F51">
+        <v>1</v>
+      </c>
+      <c r="G51">
         <v>4</v>
       </c>
-      <c r="G51">
-        <v>0</v>
-      </c>
       <c r="H51">
         <v>0</v>
       </c>
@@ -2462,12 +2714,15 @@
         <v>0</v>
       </c>
       <c r="K51">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L51">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M51">
+        <v>2</v>
+      </c>
+      <c r="N51">
         <v>0</v>
       </c>
     </row>
@@ -2475,8 +2730,10 @@
       <c r="A52">
         <v>150</v>
       </c>
-      <c r="B52">
-        <v>0</v>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Guter Plan. Und doch ist es für niemanden einfach, dem Bösen zu begegnen.</t>
+        </is>
       </c>
       <c r="C52">
         <v>0</v>
@@ -2488,10 +2745,10 @@
         <v>0</v>
       </c>
       <c r="F52">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G52">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H52">
         <v>0</v>
@@ -2506,9 +2763,12 @@
         <v>0</v>
       </c>
       <c r="L52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M52">
+        <v>1</v>
+      </c>
+      <c r="N52">
         <v>0</v>
       </c>
     </row>

</xml_diff>